<commit_message>
Candidate 2 (part): pricing entitlements and Business 2h scenario; sign-in risk explanation; Arabic workbook with not-found strings; complete numbered findings list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdiQ6L7bko35tTzSeUxyEb
</commit_message>
<xml_diff>
--- a/docs/readiness/ConversaFlow-Arabic-Review.xlsx
+++ b/docs/readiness/ConversaFlow-Arabic-Review.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Review!$A$1:$L$102</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Review!$A$1:$L$105</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="576" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="368">
   <si>
     <t xml:space="preserve">ConversaFlow — Arabic wording review</t>
   </si>
@@ -579,6 +579,33 @@
   </si>
   <si>
     <t xml:space="preserve">اختر كلمة مرور جديدة</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page not found</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notFound.body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The page you are looking for does not exist or has moved.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الصفحة التي تبحث عنها غير موجودة أو تم نقلها.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notFound.home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Go to sign-in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الانتقال إلى تسجيل الدخول</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notFound.title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الصفحة غير موجودة</t>
   </si>
   <si>
     <t xml:space="preserve">All app screens</t>
@@ -2050,7 +2077,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3353,7 +3380,7 @@
       </c>
       <c r="L44" s="19"/>
     </row>
-    <row r="45" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="n">
         <v>44</v>
       </c>
@@ -3361,22 +3388,20 @@
         <v>173</v>
       </c>
       <c r="C45" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="D45" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="D45" s="14" t="s">
+      <c r="E45" s="13" t="s">
         <v>175</v>
-      </c>
-      <c r="E45" s="13" t="s">
-        <v>176</v>
       </c>
       <c r="F45" s="15" t="s">
         <v>176</v>
       </c>
       <c r="G45" s="16"/>
       <c r="H45" s="17"/>
-      <c r="I45" s="20" t="s">
-        <v>177</v>
-      </c>
+      <c r="I45" s="16"/>
       <c r="J45" s="13"/>
       <c r="K45" s="18" t="str">
         <f aca="false">IF(G45="","To review",IF(AND(G45="Change",H45=""),"Add corrected text",IF(AND(H45&lt;&gt;"",J45&lt;&gt;"",ISERROR(SEARCH(J45,H45))),"Keep "&amp;J45,"")))</f>
@@ -3384,7 +3409,7 @@
       </c>
       <c r="L45" s="19"/>
     </row>
-    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="n">
         <v>45</v>
       </c>
@@ -3392,16 +3417,16 @@
         <v>173</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>174</v>
+        <v>110</v>
       </c>
       <c r="D46" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="E46" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="E46" s="13" t="s">
+      <c r="F46" s="15" t="s">
         <v>179</v>
-      </c>
-      <c r="F46" s="15" t="s">
-        <v>180</v>
       </c>
       <c r="G46" s="16"/>
       <c r="H46" s="17"/>
@@ -3413,7 +3438,7 @@
       </c>
       <c r="L46" s="19"/>
     </row>
-    <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="n">
         <v>46</v>
       </c>
@@ -3421,22 +3446,20 @@
         <v>173</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>174</v>
+        <v>110</v>
       </c>
       <c r="D47" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="E47" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="F47" s="15" t="s">
         <v>181</v>
-      </c>
-      <c r="E47" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="F47" s="15" t="s">
-        <v>183</v>
       </c>
       <c r="G47" s="16"/>
       <c r="H47" s="17"/>
-      <c r="I47" s="20" t="s">
-        <v>184</v>
-      </c>
+      <c r="I47" s="16"/>
       <c r="J47" s="13"/>
       <c r="K47" s="18" t="str">
         <f aca="false">IF(G47="","To review",IF(AND(G47="Change",H47=""),"Add corrected text",IF(AND(H47&lt;&gt;"",J47&lt;&gt;"",ISERROR(SEARCH(J47,H47))),"Keep "&amp;J47,"")))</f>
@@ -3449,23 +3472,25 @@
         <v>47</v>
       </c>
       <c r="B48" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D48" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="E48" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="E48" s="13" t="s">
-        <v>186</v>
-      </c>
       <c r="F48" s="15" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G48" s="16"/>
       <c r="H48" s="17"/>
-      <c r="I48" s="16"/>
+      <c r="I48" s="20" t="s">
+        <v>186</v>
+      </c>
       <c r="J48" s="13"/>
       <c r="K48" s="18" t="str">
         <f aca="false">IF(G48="","To review",IF(AND(G48="Change",H48=""),"Add corrected text",IF(AND(H48&lt;&gt;"",J48&lt;&gt;"",ISERROR(SEARCH(J48,H48))),"Keep "&amp;J48,"")))</f>
@@ -3478,19 +3503,19 @@
         <v>48</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D49" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="E49" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="E49" s="13" t="s">
+      <c r="F49" s="15" t="s">
         <v>189</v>
-      </c>
-      <c r="F49" s="15" t="s">
-        <v>190</v>
       </c>
       <c r="G49" s="16"/>
       <c r="H49" s="17"/>
@@ -3507,23 +3532,25 @@
         <v>49</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D50" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="E50" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="E50" s="13" t="s">
+      <c r="F50" s="15" t="s">
         <v>192</v>
-      </c>
-      <c r="F50" s="15" t="s">
-        <v>193</v>
       </c>
       <c r="G50" s="16"/>
       <c r="H50" s="17"/>
-      <c r="I50" s="16"/>
+      <c r="I50" s="20" t="s">
+        <v>193</v>
+      </c>
       <c r="J50" s="13"/>
       <c r="K50" s="18" t="str">
         <f aca="false">IF(G50="","To review",IF(AND(G50="Change",H50=""),"Add corrected text",IF(AND(H50&lt;&gt;"",J50&lt;&gt;"",ISERROR(SEARCH(J50,H50))),"Keep "&amp;J50,"")))</f>
@@ -3536,10 +3563,10 @@
         <v>50</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D51" s="14" t="s">
         <v>194</v>
@@ -3565,10 +3592,10 @@
         <v>51</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D52" s="14" t="s">
         <v>197</v>
@@ -3594,10 +3621,10 @@
         <v>52</v>
       </c>
       <c r="B53" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D53" s="14" t="s">
         <v>200</v>
@@ -3623,10 +3650,10 @@
         <v>53</v>
       </c>
       <c r="B54" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D54" s="14" t="s">
         <v>203</v>
@@ -3652,10 +3679,10 @@
         <v>54</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D55" s="14" t="s">
         <v>206</v>
@@ -3681,10 +3708,10 @@
         <v>55</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D56" s="14" t="s">
         <v>209</v>
@@ -3710,10 +3737,10 @@
         <v>56</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D57" s="14" t="s">
         <v>212</v>
@@ -3739,10 +3766,10 @@
         <v>57</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D58" s="14" t="s">
         <v>215</v>
@@ -3768,10 +3795,10 @@
         <v>58</v>
       </c>
       <c r="B59" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D59" s="14" t="s">
         <v>218</v>
@@ -3797,10 +3824,10 @@
         <v>59</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D60" s="14" t="s">
         <v>221</v>
@@ -3826,10 +3853,10 @@
         <v>60</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D61" s="14" t="s">
         <v>224</v>
@@ -3855,10 +3882,10 @@
         <v>61</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D62" s="14" t="s">
         <v>227</v>
@@ -3884,10 +3911,10 @@
         <v>62</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>210</v>
+        <v>182</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D63" s="14" t="s">
         <v>230</v>
@@ -3913,10 +3940,10 @@
         <v>63</v>
       </c>
       <c r="B64" s="13" t="s">
-        <v>210</v>
+        <v>182</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D64" s="14" t="s">
         <v>233</v>
@@ -3942,10 +3969,10 @@
         <v>64</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>210</v>
+        <v>182</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D65" s="14" t="s">
         <v>236</v>
@@ -3971,10 +3998,10 @@
         <v>65</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D66" s="14" t="s">
         <v>239</v>
@@ -4000,10 +4027,10 @@
         <v>66</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D67" s="14" t="s">
         <v>242</v>
@@ -4029,10 +4056,10 @@
         <v>67</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D68" s="14" t="s">
         <v>245</v>
@@ -4058,10 +4085,10 @@
         <v>68</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D69" s="14" t="s">
         <v>248</v>
@@ -4087,10 +4114,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D70" s="14" t="s">
         <v>251</v>
@@ -4103,12 +4130,8 @@
       </c>
       <c r="G70" s="16"/>
       <c r="H70" s="17"/>
-      <c r="I70" s="20" t="s">
-        <v>254</v>
-      </c>
-      <c r="J70" s="13" t="s">
-        <v>255</v>
-      </c>
+      <c r="I70" s="16"/>
+      <c r="J70" s="13"/>
       <c r="K70" s="18" t="str">
         <f aca="false">IF(G70="","To review",IF(AND(G70="Change",H70=""),"Add corrected text",IF(AND(H70&lt;&gt;"",J70&lt;&gt;"",ISERROR(SEARCH(J70,H70))),"Keep "&amp;J70,"")))</f>
         <v>To review</v>
@@ -4120,28 +4143,24 @@
         <v>70</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="D71" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="E71" s="13" t="s">
+        <v>255</v>
+      </c>
+      <c r="F71" s="15" t="s">
         <v>256</v>
-      </c>
-      <c r="E71" s="13" t="s">
-        <v>257</v>
-      </c>
-      <c r="F71" s="15" t="s">
-        <v>258</v>
       </c>
       <c r="G71" s="16"/>
       <c r="H71" s="17"/>
-      <c r="I71" s="20" t="s">
-        <v>259</v>
-      </c>
-      <c r="J71" s="13" t="s">
-        <v>260</v>
-      </c>
+      <c r="I71" s="16"/>
+      <c r="J71" s="13"/>
       <c r="K71" s="18" t="str">
         <f aca="false">IF(G71="","To review",IF(AND(G71="Change",H71=""),"Add corrected text",IF(AND(H71&lt;&gt;"",J71&lt;&gt;"",ISERROR(SEARCH(J71,H71))),"Keep "&amp;J71,"")))</f>
         <v>To review</v>
@@ -4153,19 +4172,19 @@
         <v>71</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>261</v>
+        <v>219</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>262</v>
+        <v>183</v>
       </c>
       <c r="D72" s="14" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="E72" s="13" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="F72" s="15" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="G72" s="16"/>
       <c r="H72" s="17"/>
@@ -4182,24 +4201,28 @@
         <v>72</v>
       </c>
       <c r="B73" s="13" t="s">
+        <v>219</v>
+      </c>
+      <c r="C73" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="D73" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="E73" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="C73" s="14" t="s">
+      <c r="F73" s="15" t="s">
         <v>262</v>
-      </c>
-      <c r="D73" s="14" t="s">
-        <v>266</v>
-      </c>
-      <c r="E73" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="F73" s="15" t="s">
-        <v>268</v>
       </c>
       <c r="G73" s="16"/>
       <c r="H73" s="17"/>
-      <c r="I73" s="16"/>
-      <c r="J73" s="13"/>
+      <c r="I73" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="J73" s="13" t="s">
+        <v>264</v>
+      </c>
       <c r="K73" s="18" t="str">
         <f aca="false">IF(G73="","To review",IF(AND(G73="Change",H73=""),"Add corrected text",IF(AND(H73&lt;&gt;"",J73&lt;&gt;"",ISERROR(SEARCH(J73,H73))),"Keep "&amp;J73,"")))</f>
         <v>To review</v>
@@ -4211,24 +4234,28 @@
         <v>73</v>
       </c>
       <c r="B74" s="13" t="s">
-        <v>261</v>
+        <v>219</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>262</v>
+        <v>183</v>
       </c>
       <c r="D74" s="14" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="E74" s="13" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="F74" s="15" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="G74" s="16"/>
       <c r="H74" s="17"/>
-      <c r="I74" s="16"/>
-      <c r="J74" s="13"/>
+      <c r="I74" s="20" t="s">
+        <v>268</v>
+      </c>
+      <c r="J74" s="13" t="s">
+        <v>269</v>
+      </c>
       <c r="K74" s="18" t="str">
         <f aca="false">IF(G74="","To review",IF(AND(G74="Change",H74=""),"Add corrected text",IF(AND(H74&lt;&gt;"",J74&lt;&gt;"",ISERROR(SEARCH(J74,H74))),"Keep "&amp;J74,"")))</f>
         <v>To review</v>
@@ -4240,10 +4267,10 @@
         <v>74</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C75" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D75" s="14" t="s">
         <v>272</v>
@@ -4269,10 +4296,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D76" s="14" t="s">
         <v>275</v>
@@ -4298,10 +4325,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D77" s="14" t="s">
         <v>278</v>
@@ -4327,10 +4354,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D78" s="14" t="s">
         <v>281</v>
@@ -4356,10 +4383,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D79" s="14" t="s">
         <v>284</v>
@@ -4385,10 +4412,10 @@
         <v>79</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D80" s="14" t="s">
         <v>287</v>
@@ -4414,10 +4441,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D81" s="14" t="s">
         <v>290</v>
@@ -4443,19 +4470,19 @@
         <v>81</v>
       </c>
       <c r="B82" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D82" s="14" t="s">
         <v>293</v>
       </c>
       <c r="E82" s="13" t="s">
-        <v>261</v>
+        <v>294</v>
       </c>
       <c r="F82" s="15" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G82" s="16"/>
       <c r="H82" s="17"/>
@@ -4472,19 +4499,19 @@
         <v>82</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C83" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D83" s="14" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F83" s="15" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G83" s="16"/>
       <c r="H83" s="17"/>
@@ -4501,19 +4528,19 @@
         <v>83</v>
       </c>
       <c r="B84" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C84" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D84" s="14" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F84" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G84" s="16"/>
       <c r="H84" s="17"/>
@@ -4530,16 +4557,16 @@
         <v>84</v>
       </c>
       <c r="B85" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C85" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D85" s="14" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E85" s="13" t="s">
-        <v>302</v>
+        <v>270</v>
       </c>
       <c r="F85" s="15" t="s">
         <v>303</v>
@@ -4559,10 +4586,10 @@
         <v>85</v>
       </c>
       <c r="B86" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C86" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D86" s="14" t="s">
         <v>304</v>
@@ -4588,10 +4615,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C87" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D87" s="14" t="s">
         <v>307</v>
@@ -4617,10 +4644,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C88" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D88" s="14" t="s">
         <v>310</v>
@@ -4646,10 +4673,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C89" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D89" s="14" t="s">
         <v>313</v>
@@ -4675,10 +4702,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C90" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D90" s="14" t="s">
         <v>316</v>
@@ -4687,7 +4714,7 @@
         <v>317</v>
       </c>
       <c r="F90" s="15" t="s">
-        <v>61</v>
+        <v>318</v>
       </c>
       <c r="G90" s="16"/>
       <c r="H90" s="17"/>
@@ -4704,19 +4731,19 @@
         <v>90</v>
       </c>
       <c r="B91" s="13" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D91" s="14" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E91" s="13" t="s">
-        <v>18</v>
+        <v>320</v>
       </c>
       <c r="F91" s="15" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="G91" s="16"/>
       <c r="H91" s="17"/>
@@ -4733,19 +4760,19 @@
         <v>91</v>
       </c>
       <c r="B92" s="13" t="s">
-        <v>228</v>
+        <v>270</v>
       </c>
       <c r="C92" s="14" t="s">
-        <v>320</v>
+        <v>271</v>
       </c>
       <c r="D92" s="14" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E92" s="13" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F92" s="15" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G92" s="16"/>
       <c r="H92" s="17"/>
@@ -4762,25 +4789,23 @@
         <v>92</v>
       </c>
       <c r="B93" s="13" t="s">
-        <v>228</v>
+        <v>270</v>
       </c>
       <c r="C93" s="14" t="s">
-        <v>320</v>
+        <v>271</v>
       </c>
       <c r="D93" s="14" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E93" s="13" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F93" s="15" t="s">
-        <v>326</v>
+        <v>61</v>
       </c>
       <c r="G93" s="16"/>
       <c r="H93" s="17"/>
-      <c r="I93" s="20" t="s">
-        <v>327</v>
-      </c>
+      <c r="I93" s="16"/>
       <c r="J93" s="13"/>
       <c r="K93" s="18" t="str">
         <f aca="false">IF(G93="","To review",IF(AND(G93="Change",H93=""),"Add corrected text",IF(AND(H93&lt;&gt;"",J93&lt;&gt;"",ISERROR(SEARCH(J93,H93))),"Keep "&amp;J93,"")))</f>
@@ -4793,19 +4818,19 @@
         <v>93</v>
       </c>
       <c r="B94" s="13" t="s">
-        <v>228</v>
+        <v>270</v>
       </c>
       <c r="C94" s="14" t="s">
-        <v>320</v>
+        <v>271</v>
       </c>
       <c r="D94" s="14" t="s">
+        <v>327</v>
+      </c>
+      <c r="E94" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F94" s="15" t="s">
         <v>328</v>
-      </c>
-      <c r="E94" s="13" t="s">
-        <v>329</v>
-      </c>
-      <c r="F94" s="15" t="s">
-        <v>330</v>
       </c>
       <c r="G94" s="16"/>
       <c r="H94" s="17"/>
@@ -4822,19 +4847,19 @@
         <v>94</v>
       </c>
       <c r="B95" s="13" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C95" s="14" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D95" s="14" t="s">
+        <v>330</v>
+      </c>
+      <c r="E95" s="13" t="s">
         <v>331</v>
       </c>
-      <c r="E95" s="13" t="s">
+      <c r="F95" s="15" t="s">
         <v>332</v>
-      </c>
-      <c r="F95" s="15" t="s">
-        <v>333</v>
       </c>
       <c r="G95" s="16"/>
       <c r="H95" s="17"/>
@@ -4851,23 +4876,25 @@
         <v>95</v>
       </c>
       <c r="B96" s="13" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C96" s="14" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D96" s="14" t="s">
+        <v>333</v>
+      </c>
+      <c r="E96" s="13" t="s">
         <v>334</v>
       </c>
-      <c r="E96" s="13" t="s">
+      <c r="F96" s="15" t="s">
         <v>335</v>
-      </c>
-      <c r="F96" s="15" t="s">
-        <v>336</v>
       </c>
       <c r="G96" s="16"/>
       <c r="H96" s="17"/>
-      <c r="I96" s="16"/>
+      <c r="I96" s="20" t="s">
+        <v>336</v>
+      </c>
       <c r="J96" s="13"/>
       <c r="K96" s="18" t="str">
         <f aca="false">IF(G96="","To review",IF(AND(G96="Change",H96=""),"Add corrected text",IF(AND(H96&lt;&gt;"",J96&lt;&gt;"",ISERROR(SEARCH(J96,H96))),"Keep "&amp;J96,"")))</f>
@@ -4880,10 +4907,10 @@
         <v>96</v>
       </c>
       <c r="B97" s="13" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C97" s="14" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D97" s="14" t="s">
         <v>337</v>
@@ -4909,10 +4936,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="13" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C98" s="14" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D98" s="14" t="s">
         <v>340</v>
@@ -4921,7 +4948,7 @@
         <v>341</v>
       </c>
       <c r="F98" s="15" t="s">
-        <v>74</v>
+        <v>342</v>
       </c>
       <c r="G98" s="16"/>
       <c r="H98" s="17"/>
@@ -4938,19 +4965,19 @@
         <v>98</v>
       </c>
       <c r="B99" s="13" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C99" s="14" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D99" s="14" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="E99" s="13" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="F99" s="15" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G99" s="16"/>
       <c r="H99" s="17"/>
@@ -4967,19 +4994,19 @@
         <v>99</v>
       </c>
       <c r="B100" s="13" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C100" s="14" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D100" s="14" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E100" s="13" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F100" s="15" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G100" s="16"/>
       <c r="H100" s="17"/>
@@ -4996,19 +5023,19 @@
         <v>100</v>
       </c>
       <c r="B101" s="13" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C101" s="14" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D101" s="14" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E101" s="13" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F101" s="15" t="s">
-        <v>350</v>
+        <v>74</v>
       </c>
       <c r="G101" s="16"/>
       <c r="H101" s="17"/>
@@ -5025,19 +5052,19 @@
         <v>101</v>
       </c>
       <c r="B102" s="13" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="C102" s="14" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="D102" s="14" t="s">
         <v>351</v>
       </c>
       <c r="E102" s="13" t="s">
-        <v>228</v>
+        <v>352</v>
       </c>
       <c r="F102" s="15" t="s">
-        <v>229</v>
+        <v>353</v>
       </c>
       <c r="G102" s="16"/>
       <c r="H102" s="17"/>
@@ -5049,9 +5076,96 @@
       </c>
       <c r="L102" s="19"/>
     </row>
+    <row r="103" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="13" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="C103" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="D103" s="14" t="s">
+        <v>354</v>
+      </c>
+      <c r="E103" s="13" t="s">
+        <v>355</v>
+      </c>
+      <c r="F103" s="15" t="s">
+        <v>356</v>
+      </c>
+      <c r="G103" s="16"/>
+      <c r="H103" s="17"/>
+      <c r="I103" s="16"/>
+      <c r="J103" s="13"/>
+      <c r="K103" s="18" t="str">
+        <f aca="false">IF(G103="","To review",IF(AND(G103="Change",H103=""),"Add corrected text",IF(AND(H103&lt;&gt;"",J103&lt;&gt;"",ISERROR(SEARCH(J103,H103))),"Keep "&amp;J103,"")))</f>
+        <v>To review</v>
+      </c>
+      <c r="L103" s="19"/>
+    </row>
+    <row r="104" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="13" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="C104" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="D104" s="14" t="s">
+        <v>357</v>
+      </c>
+      <c r="E104" s="13" t="s">
+        <v>358</v>
+      </c>
+      <c r="F104" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="G104" s="16"/>
+      <c r="H104" s="17"/>
+      <c r="I104" s="16"/>
+      <c r="J104" s="13"/>
+      <c r="K104" s="18" t="str">
+        <f aca="false">IF(G104="","To review",IF(AND(G104="Change",H104=""),"Add corrected text",IF(AND(H104&lt;&gt;"",J104&lt;&gt;"",ISERROR(SEARCH(J104,H104))),"Keep "&amp;J104,"")))</f>
+        <v>To review</v>
+      </c>
+      <c r="L104" s="19"/>
+    </row>
+    <row r="105" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="13" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="C105" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="D105" s="14" t="s">
+        <v>360</v>
+      </c>
+      <c r="E105" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="F105" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="G105" s="16"/>
+      <c r="H105" s="17"/>
+      <c r="I105" s="16"/>
+      <c r="J105" s="13"/>
+      <c r="K105" s="18" t="str">
+        <f aca="false">IF(G105="","To review",IF(AND(G105="Change",H105=""),"Add corrected text",IF(AND(H105&lt;&gt;"",J105&lt;&gt;"",ISERROR(SEARCH(J105,H105))),"Keep "&amp;J105,"")))</f>
+        <v>To review</v>
+      </c>
+      <c r="L105" s="19"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L102"/>
-  <conditionalFormatting sqref="A2:L102">
+  <autoFilter ref="A1:L105"/>
+  <conditionalFormatting sqref="A2:L105">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$G2="Change"</formula>
     </cfRule>
@@ -5060,11 +5174,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Choose OK, Change or Question." errorStyle="stop" errorTitle="Your verdict" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G102" type="list">
+    <dataValidation allowBlank="true" error="Choose OK, Change or Question." errorStyle="stop" errorTitle="Your verdict" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G105" type="list">
       <formula1>"OK,Change,Question"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L102" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L105" type="list">
       <formula1>"Applied,Not needed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5086,7 +5200,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -5098,25 +5212,25 @@
         <v>17</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>352</v>
+        <v>361</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>353</v>
+        <v>362</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>354</v>
+        <v>363</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>356</v>
+        <v>365</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5124,23 +5238,23 @@
         <v>23</v>
       </c>
       <c r="B2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A2)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2)</f>
         <v>23</v>
       </c>
       <c r="C2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A2,Review!$G$2:$G$102,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A2,Review!$G$2:$G$102,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
       <c r="E2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A2,Review!$G$2:$G$102,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
       <c r="F2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A2,Review!$G$2:$G$102,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
       <c r="G2" s="21" t="n">
@@ -5148,7 +5262,7 @@
         <v>23</v>
       </c>
       <c r="H2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A2,Review!$L$2:$L$102,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$L$2:$L$105,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5157,23 +5271,23 @@
         <v>109</v>
       </c>
       <c r="B3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A3)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3)</f>
         <v>9</v>
       </c>
       <c r="C3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A3,Review!$G$2:$G$102,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A3,Review!$G$2:$G$102,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
       <c r="E3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A3,Review!$G$2:$G$102,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
       <c r="F3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A3,Review!$G$2:$G$102,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
       <c r="G3" s="21" t="n">
@@ -5181,7 +5295,7 @@
         <v>9</v>
       </c>
       <c r="H3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A3,Review!$L$2:$L$102,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$L$2:$L$105,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5190,23 +5304,23 @@
         <v>137</v>
       </c>
       <c r="B4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A4)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4)</f>
         <v>3</v>
       </c>
       <c r="C4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A4,Review!$G$2:$G$102,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A4,Review!$G$2:$G$102,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
       <c r="E4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A4,Review!$G$2:$G$102,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
       <c r="F4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A4,Review!$G$2:$G$102,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
       <c r="G4" s="21" t="n">
@@ -5214,7 +5328,7 @@
         <v>3</v>
       </c>
       <c r="H4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A4,Review!$L$2:$L$102,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$L$2:$L$105,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5223,23 +5337,23 @@
         <v>147</v>
       </c>
       <c r="B5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A5)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5)</f>
         <v>3</v>
       </c>
       <c r="C5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A5,Review!$G$2:$G$102,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A5,Review!$G$2:$G$102,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
       <c r="E5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A5,Review!$G$2:$G$102,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
       <c r="F5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A5,Review!$G$2:$G$102,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
       <c r="G5" s="21" t="n">
@@ -5247,7 +5361,7 @@
         <v>3</v>
       </c>
       <c r="H5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A5,Review!$L$2:$L$102,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$L$2:$L$105,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5256,23 +5370,23 @@
         <v>157</v>
       </c>
       <c r="B6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A6)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6)</f>
         <v>5</v>
       </c>
       <c r="C6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A6,Review!$G$2:$G$102,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A6,Review!$G$2:$G$102,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
       <c r="E6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A6,Review!$G$2:$G$102,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
       <c r="F6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A6,Review!$G$2:$G$102,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
       <c r="G6" s="21" t="n">
@@ -5280,7 +5394,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A6,Review!$L$2:$L$102,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$L$2:$L$105,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5289,163 +5403,196 @@
         <v>173</v>
       </c>
       <c r="B7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A7)</f>
-        <v>18</v>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7)</f>
+        <v>3</v>
       </c>
       <c r="C7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A7,Review!$G$2:$G$102,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A7,Review!$G$2:$G$102,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
       <c r="E7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A7,Review!$G$2:$G$102,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
       <c r="F7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A7,Review!$G$2:$G$102,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
       <c r="G7" s="21" t="n">
         <f aca="false">B7-C7</f>
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="H7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A7,Review!$L$2:$L$102,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$L$2:$L$105,"Applied")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>210</v>
+        <v>182</v>
       </c>
       <c r="B8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A8)</f>
-        <v>9</v>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8)</f>
+        <v>18</v>
       </c>
       <c r="C8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A8,Review!$G$2:$G$102,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A8,Review!$G$2:$G$102,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
       <c r="E8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A8,Review!$G$2:$G$102,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
       <c r="F8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A8,Review!$G$2:$G$102,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
       <c r="G8" s="21" t="n">
         <f aca="false">B8-C8</f>
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="H8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A8,Review!$L$2:$L$102,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$L$2:$L$105,"Applied")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>261</v>
+        <v>219</v>
       </c>
       <c r="B9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A9)</f>
-        <v>20</v>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9)</f>
+        <v>9</v>
       </c>
       <c r="C9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A9,Review!$G$2:$G$102,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A9,Review!$G$2:$G$102,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
       <c r="E9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A9,Review!$G$2:$G$102,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
       <c r="F9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A9,Review!$G$2:$G$102,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
       <c r="G9" s="21" t="n">
         <f aca="false">B9-C9</f>
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="H9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A9,Review!$L$2:$L$102,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$L$2:$L$105,"Applied")</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>228</v>
+        <v>270</v>
       </c>
       <c r="B10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A10)</f>
-        <v>11</v>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10)</f>
+        <v>20</v>
       </c>
       <c r="C10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A10,Review!$G$2:$G$102,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A10,Review!$G$2:$G$102,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
       <c r="E10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A10,Review!$G$2:$G$102,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
       <c r="F10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A10,Review!$G$2:$G$102,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
       <c r="G10" s="21" t="n">
         <f aca="false">B10-C10</f>
+        <v>20</v>
+      </c>
+      <c r="H10" s="21" t="n">
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$L$2:$L$105,"Applied")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
+        <v>237</v>
+      </c>
+      <c r="B11" s="21" t="n">
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11)</f>
         <v>11</v>
       </c>
-      <c r="H10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$102,A10,Review!$L$2:$L$102,"Applied")</f>
+      <c r="C11" s="21" t="n">
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$G$2:$G$105,"&lt;&gt;")</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
-        <v>358</v>
-      </c>
-      <c r="B11" s="22" t="n">
-        <f aca="false">SUM(B2:B10)</f>
-        <v>101</v>
-      </c>
-      <c r="C11" s="22" t="n">
-        <f aca="false">SUM(C2:C10)</f>
+      <c r="D11" s="21" t="n">
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$G$2:$G$105,"OK")</f>
         <v>0</v>
       </c>
-      <c r="D11" s="22" t="n">
-        <f aca="false">SUM(D2:D10)</f>
+      <c r="E11" s="21" t="n">
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$G$2:$G$105,"Change")</f>
         <v>0</v>
       </c>
-      <c r="E11" s="22" t="n">
-        <f aca="false">SUM(E2:E10)</f>
+      <c r="F11" s="21" t="n">
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$G$2:$G$105,"Question")</f>
         <v>0</v>
       </c>
-      <c r="F11" s="22" t="n">
-        <f aca="false">SUM(F2:F10)</f>
+      <c r="G11" s="21" t="n">
+        <f aca="false">B11-C11</f>
+        <v>11</v>
+      </c>
+      <c r="H11" s="21" t="n">
+        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$L$2:$L$105,"Applied")</f>
         <v>0</v>
       </c>
-      <c r="G11" s="22" t="n">
-        <f aca="false">SUM(G2:G10)</f>
-        <v>101</v>
-      </c>
-      <c r="H11" s="22" t="n">
-        <f aca="false">SUM(H2:H10)</f>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="22" t="s">
+        <v>367</v>
+      </c>
+      <c r="B12" s="22" t="n">
+        <f aca="false">SUM(B2:B11)</f>
+        <v>104</v>
+      </c>
+      <c r="C12" s="22" t="n">
+        <f aca="false">SUM(C2:C11)</f>
+        <v>0</v>
+      </c>
+      <c r="D12" s="22" t="n">
+        <f aca="false">SUM(D2:D11)</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="22" t="n">
+        <f aca="false">SUM(E2:E11)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="22" t="n">
+        <f aca="false">SUM(F2:F11)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="22" t="n">
+        <f aca="false">SUM(G2:G11)</f>
+        <v>104</v>
+      </c>
+      <c r="H12" s="22" t="n">
+        <f aca="false">SUM(H2:H11)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Candidate 3: M7 email-confirmed authenticator (0016), M8 two-person audited reset (0017), M9 72-hour revocable pilot invitations; CI guard for privileged pilot/override writers; client.ts code owner; unsupported-browser notice and Firefox/WebKit CI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AdiQ6L7bko35tTzSeUxyEb
</commit_message>
<xml_diff>
--- a/docs/readiness/ConversaFlow-Arabic-Review.xlsx
+++ b/docs/readiness/ConversaFlow-Arabic-Review.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Review!$A$1:$L$105</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Review!$A$1:$L$106</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="371">
   <si>
     <t xml:space="preserve">ConversaFlow — Arabic wording review</t>
   </si>
@@ -622,6 +622,15 @@
   </si>
   <si>
     <t xml:space="preserve">Kept in Latin script on purpose (brand lockup). Check only; no translation expected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">browser.unsupported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Your browser is too old for ConversaFlow. Please update to a recent Safari (iOS 16.4 or later), Chrome, Edge or Firefox.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">متصفحك قديم ولا يدعم ConversaFlow. يُرجى التحديث إلى إصدار حديث من Safari (iOS 16.4 أو أحدث) أو Chrome أو Edge أو Firefox.</t>
   </si>
   <si>
     <t xml:space="preserve">common.error</t>
@@ -2077,7 +2086,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3498,7 +3507,7 @@
       </c>
       <c r="L48" s="19"/>
     </row>
-    <row r="49" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="n">
         <v>48</v>
       </c>
@@ -3548,9 +3557,7 @@
       </c>
       <c r="G50" s="16"/>
       <c r="H50" s="17"/>
-      <c r="I50" s="20" t="s">
-        <v>193</v>
-      </c>
+      <c r="I50" s="16"/>
       <c r="J50" s="13"/>
       <c r="K50" s="18" t="str">
         <f aca="false">IF(G50="","To review",IF(AND(G50="Change",H50=""),"Add corrected text",IF(AND(H50&lt;&gt;"",J50&lt;&gt;"",ISERROR(SEARCH(J50,H50))),"Keep "&amp;J50,"")))</f>
@@ -3569,17 +3576,19 @@
         <v>183</v>
       </c>
       <c r="D51" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="E51" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="E51" s="13" t="s">
+      <c r="F51" s="15" t="s">
         <v>195</v>
-      </c>
-      <c r="F51" s="15" t="s">
-        <v>196</v>
       </c>
       <c r="G51" s="16"/>
       <c r="H51" s="17"/>
-      <c r="I51" s="16"/>
+      <c r="I51" s="20" t="s">
+        <v>196</v>
+      </c>
       <c r="J51" s="13"/>
       <c r="K51" s="18" t="str">
         <f aca="false">IF(G51="","To review",IF(AND(G51="Change",H51=""),"Add corrected text",IF(AND(H51&lt;&gt;"",J51&lt;&gt;"",ISERROR(SEARCH(J51,H51))),"Keep "&amp;J51,"")))</f>
@@ -3998,7 +4007,7 @@
         <v>65</v>
       </c>
       <c r="B66" s="13" t="s">
-        <v>219</v>
+        <v>182</v>
       </c>
       <c r="C66" s="14" t="s">
         <v>183</v>
@@ -4027,7 +4036,7 @@
         <v>66</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C67" s="14" t="s">
         <v>183</v>
@@ -4056,7 +4065,7 @@
         <v>67</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C68" s="14" t="s">
         <v>183</v>
@@ -4085,7 +4094,7 @@
         <v>68</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C69" s="14" t="s">
         <v>183</v>
@@ -4114,7 +4123,7 @@
         <v>69</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C70" s="14" t="s">
         <v>183</v>
@@ -4143,7 +4152,7 @@
         <v>70</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C71" s="14" t="s">
         <v>183</v>
@@ -4172,7 +4181,7 @@
         <v>71</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C72" s="14" t="s">
         <v>183</v>
@@ -4201,7 +4210,7 @@
         <v>72</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C73" s="14" t="s">
         <v>183</v>
@@ -4217,12 +4226,8 @@
       </c>
       <c r="G73" s="16"/>
       <c r="H73" s="17"/>
-      <c r="I73" s="20" t="s">
-        <v>263</v>
-      </c>
-      <c r="J73" s="13" t="s">
-        <v>264</v>
-      </c>
+      <c r="I73" s="16"/>
+      <c r="J73" s="13"/>
       <c r="K73" s="18" t="str">
         <f aca="false">IF(G73="","To review",IF(AND(G73="Change",H73=""),"Add corrected text",IF(AND(H73&lt;&gt;"",J73&lt;&gt;"",ISERROR(SEARCH(J73,H73))),"Keep "&amp;J73,"")))</f>
         <v>To review</v>
@@ -4234,27 +4239,27 @@
         <v>73</v>
       </c>
       <c r="B74" s="13" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C74" s="14" t="s">
         <v>183</v>
       </c>
       <c r="D74" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="E74" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="F74" s="15" t="s">
         <v>265</v>
-      </c>
-      <c r="E74" s="13" t="s">
-        <v>266</v>
-      </c>
-      <c r="F74" s="15" t="s">
-        <v>267</v>
       </c>
       <c r="G74" s="16"/>
       <c r="H74" s="17"/>
       <c r="I74" s="20" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="J74" s="13" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="K74" s="18" t="str">
         <f aca="false">IF(G74="","To review",IF(AND(G74="Change",H74=""),"Add corrected text",IF(AND(H74&lt;&gt;"",J74&lt;&gt;"",ISERROR(SEARCH(J74,H74))),"Keep "&amp;J74,"")))</f>
@@ -4267,24 +4272,28 @@
         <v>74</v>
       </c>
       <c r="B75" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="C75" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="D75" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="E75" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="F75" s="15" t="s">
         <v>270</v>
-      </c>
-      <c r="C75" s="14" t="s">
-        <v>271</v>
-      </c>
-      <c r="D75" s="14" t="s">
-        <v>272</v>
-      </c>
-      <c r="E75" s="13" t="s">
-        <v>273</v>
-      </c>
-      <c r="F75" s="15" t="s">
-        <v>274</v>
       </c>
       <c r="G75" s="16"/>
       <c r="H75" s="17"/>
-      <c r="I75" s="16"/>
-      <c r="J75" s="13"/>
+      <c r="I75" s="20" t="s">
+        <v>271</v>
+      </c>
+      <c r="J75" s="13" t="s">
+        <v>272</v>
+      </c>
       <c r="K75" s="18" t="str">
         <f aca="false">IF(G75="","To review",IF(AND(G75="Change",H75=""),"Add corrected text",IF(AND(H75&lt;&gt;"",J75&lt;&gt;"",ISERROR(SEARCH(J75,H75))),"Keep "&amp;J75,"")))</f>
         <v>To review</v>
@@ -4296,10 +4305,10 @@
         <v>75</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D76" s="14" t="s">
         <v>275</v>
@@ -4325,10 +4334,10 @@
         <v>76</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D77" s="14" t="s">
         <v>278</v>
@@ -4354,10 +4363,10 @@
         <v>77</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C78" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D78" s="14" t="s">
         <v>281</v>
@@ -4383,10 +4392,10 @@
         <v>78</v>
       </c>
       <c r="B79" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C79" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D79" s="14" t="s">
         <v>284</v>
@@ -4412,10 +4421,10 @@
         <v>79</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C80" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D80" s="14" t="s">
         <v>287</v>
@@ -4441,10 +4450,10 @@
         <v>80</v>
       </c>
       <c r="B81" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C81" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D81" s="14" t="s">
         <v>290</v>
@@ -4470,10 +4479,10 @@
         <v>81</v>
       </c>
       <c r="B82" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C82" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D82" s="14" t="s">
         <v>293</v>
@@ -4499,10 +4508,10 @@
         <v>82</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C83" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D83" s="14" t="s">
         <v>296</v>
@@ -4528,10 +4537,10 @@
         <v>83</v>
       </c>
       <c r="B84" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C84" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D84" s="14" t="s">
         <v>299</v>
@@ -4557,19 +4566,19 @@
         <v>84</v>
       </c>
       <c r="B85" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C85" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D85" s="14" t="s">
         <v>302</v>
       </c>
       <c r="E85" s="13" t="s">
-        <v>270</v>
+        <v>303</v>
       </c>
       <c r="F85" s="15" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="G85" s="16"/>
       <c r="H85" s="17"/>
@@ -4586,16 +4595,16 @@
         <v>85</v>
       </c>
       <c r="B86" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C86" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D86" s="14" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E86" s="13" t="s">
-        <v>305</v>
+        <v>273</v>
       </c>
       <c r="F86" s="15" t="s">
         <v>306</v>
@@ -4615,10 +4624,10 @@
         <v>86</v>
       </c>
       <c r="B87" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C87" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D87" s="14" t="s">
         <v>307</v>
@@ -4644,10 +4653,10 @@
         <v>87</v>
       </c>
       <c r="B88" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C88" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D88" s="14" t="s">
         <v>310</v>
@@ -4673,10 +4682,10 @@
         <v>88</v>
       </c>
       <c r="B89" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C89" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D89" s="14" t="s">
         <v>313</v>
@@ -4702,10 +4711,10 @@
         <v>89</v>
       </c>
       <c r="B90" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C90" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D90" s="14" t="s">
         <v>316</v>
@@ -4731,10 +4740,10 @@
         <v>90</v>
       </c>
       <c r="B91" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D91" s="14" t="s">
         <v>319</v>
@@ -4760,10 +4769,10 @@
         <v>91</v>
       </c>
       <c r="B92" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C92" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D92" s="14" t="s">
         <v>322</v>
@@ -4789,10 +4798,10 @@
         <v>92</v>
       </c>
       <c r="B93" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C93" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D93" s="14" t="s">
         <v>325</v>
@@ -4801,7 +4810,7 @@
         <v>326</v>
       </c>
       <c r="F93" s="15" t="s">
-        <v>61</v>
+        <v>327</v>
       </c>
       <c r="G93" s="16"/>
       <c r="H93" s="17"/>
@@ -4818,19 +4827,19 @@
         <v>93</v>
       </c>
       <c r="B94" s="13" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C94" s="14" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D94" s="14" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E94" s="13" t="s">
-        <v>18</v>
+        <v>329</v>
       </c>
       <c r="F94" s="15" t="s">
-        <v>328</v>
+        <v>61</v>
       </c>
       <c r="G94" s="16"/>
       <c r="H94" s="17"/>
@@ -4847,19 +4856,19 @@
         <v>94</v>
       </c>
       <c r="B95" s="13" t="s">
-        <v>237</v>
+        <v>273</v>
       </c>
       <c r="C95" s="14" t="s">
-        <v>329</v>
+        <v>274</v>
       </c>
       <c r="D95" s="14" t="s">
         <v>330</v>
       </c>
       <c r="E95" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F95" s="15" t="s">
         <v>331</v>
-      </c>
-      <c r="F95" s="15" t="s">
-        <v>332</v>
       </c>
       <c r="G95" s="16"/>
       <c r="H95" s="17"/>
@@ -4876,10 +4885,10 @@
         <v>95</v>
       </c>
       <c r="B96" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C96" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D96" s="14" t="s">
         <v>333</v>
@@ -4892,9 +4901,7 @@
       </c>
       <c r="G96" s="16"/>
       <c r="H96" s="17"/>
-      <c r="I96" s="20" t="s">
-        <v>336</v>
-      </c>
+      <c r="I96" s="16"/>
       <c r="J96" s="13"/>
       <c r="K96" s="18" t="str">
         <f aca="false">IF(G96="","To review",IF(AND(G96="Change",H96=""),"Add corrected text",IF(AND(H96&lt;&gt;"",J96&lt;&gt;"",ISERROR(SEARCH(J96,H96))),"Keep "&amp;J96,"")))</f>
@@ -4907,23 +4914,25 @@
         <v>96</v>
       </c>
       <c r="B97" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C97" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D97" s="14" t="s">
+        <v>336</v>
+      </c>
+      <c r="E97" s="13" t="s">
         <v>337</v>
       </c>
-      <c r="E97" s="13" t="s">
+      <c r="F97" s="15" t="s">
         <v>338</v>
-      </c>
-      <c r="F97" s="15" t="s">
-        <v>339</v>
       </c>
       <c r="G97" s="16"/>
       <c r="H97" s="17"/>
-      <c r="I97" s="16"/>
+      <c r="I97" s="20" t="s">
+        <v>339</v>
+      </c>
       <c r="J97" s="13"/>
       <c r="K97" s="18" t="str">
         <f aca="false">IF(G97="","To review",IF(AND(G97="Change",H97=""),"Add corrected text",IF(AND(H97&lt;&gt;"",J97&lt;&gt;"",ISERROR(SEARCH(J97,H97))),"Keep "&amp;J97,"")))</f>
@@ -4936,10 +4945,10 @@
         <v>97</v>
       </c>
       <c r="B98" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C98" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D98" s="14" t="s">
         <v>340</v>
@@ -4965,10 +4974,10 @@
         <v>98</v>
       </c>
       <c r="B99" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C99" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D99" s="14" t="s">
         <v>343</v>
@@ -4994,10 +5003,10 @@
         <v>99</v>
       </c>
       <c r="B100" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C100" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D100" s="14" t="s">
         <v>346</v>
@@ -5023,10 +5032,10 @@
         <v>100</v>
       </c>
       <c r="B101" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C101" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D101" s="14" t="s">
         <v>349</v>
@@ -5035,7 +5044,7 @@
         <v>350</v>
       </c>
       <c r="F101" s="15" t="s">
-        <v>74</v>
+        <v>351</v>
       </c>
       <c r="G101" s="16"/>
       <c r="H101" s="17"/>
@@ -5052,19 +5061,19 @@
         <v>101</v>
       </c>
       <c r="B102" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C102" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D102" s="14" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="E102" s="13" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="F102" s="15" t="s">
-        <v>353</v>
+        <v>74</v>
       </c>
       <c r="G102" s="16"/>
       <c r="H102" s="17"/>
@@ -5081,10 +5090,10 @@
         <v>102</v>
       </c>
       <c r="B103" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C103" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D103" s="14" t="s">
         <v>354</v>
@@ -5110,10 +5119,10 @@
         <v>103</v>
       </c>
       <c r="B104" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C104" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D104" s="14" t="s">
         <v>357</v>
@@ -5139,19 +5148,19 @@
         <v>104</v>
       </c>
       <c r="B105" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="C105" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D105" s="14" t="s">
         <v>360</v>
       </c>
       <c r="E105" s="13" t="s">
-        <v>237</v>
+        <v>361</v>
       </c>
       <c r="F105" s="15" t="s">
-        <v>238</v>
+        <v>362</v>
       </c>
       <c r="G105" s="16"/>
       <c r="H105" s="17"/>
@@ -5163,9 +5172,38 @@
       </c>
       <c r="L105" s="19"/>
     </row>
+    <row r="106" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="13" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="C106" s="14" t="s">
+        <v>332</v>
+      </c>
+      <c r="D106" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="E106" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="F106" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="G106" s="16"/>
+      <c r="H106" s="17"/>
+      <c r="I106" s="16"/>
+      <c r="J106" s="13"/>
+      <c r="K106" s="18" t="str">
+        <f aca="false">IF(G106="","To review",IF(AND(G106="Change",H106=""),"Add corrected text",IF(AND(H106&lt;&gt;"",J106&lt;&gt;"",ISERROR(SEARCH(J106,H106))),"Keep "&amp;J106,"")))</f>
+        <v>To review</v>
+      </c>
+      <c r="L106" s="19"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L105"/>
-  <conditionalFormatting sqref="A2:L105">
+  <autoFilter ref="A1:L106"/>
+  <conditionalFormatting sqref="A2:L106">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$G2="Change"</formula>
     </cfRule>
@@ -5174,11 +5212,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" error="Choose OK, Change or Question." errorStyle="stop" errorTitle="Your verdict" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G105" type="list">
+    <dataValidation allowBlank="true" error="Choose OK, Change or Question." errorStyle="stop" errorTitle="Your verdict" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G2:G106" type="list">
       <formula1>"OK,Change,Question"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L105" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L2:L106" type="list">
       <formula1>"Applied,Not needed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -5212,25 +5250,25 @@
         <v>17</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>26</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5238,23 +5276,23 @@
         <v>23</v>
       </c>
       <c r="B2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A2)</f>
         <v>23</v>
       </c>
       <c r="C2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A2,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A2,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A2,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A2,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G2" s="21" t="n">
@@ -5262,7 +5300,7 @@
         <v>23</v>
       </c>
       <c r="H2" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A2,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A2,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5271,23 +5309,23 @@
         <v>109</v>
       </c>
       <c r="B3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A3)</f>
         <v>9</v>
       </c>
       <c r="C3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A3,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A3,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A3,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A3,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G3" s="21" t="n">
@@ -5295,7 +5333,7 @@
         <v>9</v>
       </c>
       <c r="H3" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A3,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A3,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5304,23 +5342,23 @@
         <v>137</v>
       </c>
       <c r="B4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A4)</f>
         <v>3</v>
       </c>
       <c r="C4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A4,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A4,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A4,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A4,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G4" s="21" t="n">
@@ -5328,7 +5366,7 @@
         <v>3</v>
       </c>
       <c r="H4" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A4,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A4,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5337,23 +5375,23 @@
         <v>147</v>
       </c>
       <c r="B5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A5)</f>
         <v>3</v>
       </c>
       <c r="C5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A5,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A5,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A5,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A5,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G5" s="21" t="n">
@@ -5361,7 +5399,7 @@
         <v>3</v>
       </c>
       <c r="H5" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A5,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A5,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5370,23 +5408,23 @@
         <v>157</v>
       </c>
       <c r="B6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A6)</f>
         <v>5</v>
       </c>
       <c r="C6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A6,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A6,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A6,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A6,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G6" s="21" t="n">
@@ -5394,7 +5432,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A6,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A6,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5403,23 +5441,23 @@
         <v>173</v>
       </c>
       <c r="B7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A7)</f>
         <v>3</v>
       </c>
       <c r="C7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A7,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A7,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A7,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A7,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G7" s="21" t="n">
@@ -5427,7 +5465,7 @@
         <v>3</v>
       </c>
       <c r="H7" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A7,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A7,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
@@ -5436,56 +5474,56 @@
         <v>182</v>
       </c>
       <c r="B8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8)</f>
-        <v>18</v>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A8)</f>
+        <v>19</v>
       </c>
       <c r="C8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A8,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A8,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A8,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A8,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G8" s="21" t="n">
         <f aca="false">B8-C8</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H8" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A8,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A8,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A9)</f>
         <v>9</v>
       </c>
       <c r="C9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A9,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A9,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A9,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A9,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G9" s="21" t="n">
@@ -5493,32 +5531,32 @@
         <v>9</v>
       </c>
       <c r="H9" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A9,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A9,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A10)</f>
         <v>20</v>
       </c>
       <c r="C10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A10,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A10,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A10,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A10,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G10" s="21" t="n">
@@ -5526,32 +5564,32 @@
         <v>20</v>
       </c>
       <c r="H10" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A10,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A10,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B11" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11)</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A11)</f>
         <v>11</v>
       </c>
       <c r="C11" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$G$2:$G$105,"&lt;&gt;")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A11,Review!$G$2:$G$106,"&lt;&gt;")</f>
         <v>0</v>
       </c>
       <c r="D11" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$G$2:$G$105,"OK")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A11,Review!$G$2:$G$106,"OK")</f>
         <v>0</v>
       </c>
       <c r="E11" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$G$2:$G$105,"Change")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A11,Review!$G$2:$G$106,"Change")</f>
         <v>0</v>
       </c>
       <c r="F11" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$G$2:$G$105,"Question")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A11,Review!$G$2:$G$106,"Question")</f>
         <v>0</v>
       </c>
       <c r="G11" s="21" t="n">
@@ -5559,17 +5597,17 @@
         <v>11</v>
       </c>
       <c r="H11" s="21" t="n">
-        <f aca="false">COUNTIFS(Review!$B$2:$B$105,A11,Review!$L$2:$L$105,"Applied")</f>
+        <f aca="false">COUNTIFS(Review!$B$2:$B$106,A11,Review!$L$2:$L$106,"Applied")</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B12" s="22" t="n">
         <f aca="false">SUM(B2:B11)</f>
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C12" s="22" t="n">
         <f aca="false">SUM(C2:C11)</f>
@@ -5589,7 +5627,7 @@
       </c>
       <c r="G12" s="22" t="n">
         <f aca="false">SUM(G2:G11)</f>
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H12" s="22" t="n">
         <f aca="false">SUM(H2:H11)</f>

</xml_diff>